<commit_message>
Add email columns to Quebec mosque list build
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013QAvGezT92hRi1LAbYSDwT
</commit_message>
<xml_diff>
--- a/quebec-mosques/quebec_mosques.xlsx
+++ b/quebec-mosques/quebec_mosques.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Mosquées QC" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mosquées QC'!$A$1:$J$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mosquées QC'!$A$1:$M$113</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J113"/>
+  <dimension ref="A1:M113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -435,9 +435,12 @@
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,17 +481,32 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>alt_email</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>website</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>source</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>email_source</t>
         </is>
       </c>
     </row>
@@ -528,21 +546,24 @@
           <t>450-750-0123</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
         <is>
           <t>https://acml-joliette.org/</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
         <is>
           <t>https://prayersconnect.com/mosques/12412579-joliette-mosque-joliette-quebec-canada</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -569,16 +590,19 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>https://esalah.com/mosques/canada/laval/laval/</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -605,16 +629,19 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>https://esalah.com/mosques/canada/laval/laval/</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -652,21 +679,24 @@
           <t>514-250-0265</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
         <is>
           <t>https://centreiqra.org/</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>https://www.mosquee-proche.com/fr/mosquee/ccmi-centre-communautaire-musulman-iqra-laval-h7v-2v5-canada/5496/</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -705,16 +735,19 @@
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>https://esalah.com/mosques/canada/laval/laval/</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -753,16 +786,19 @@
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>https://islammessage.org/en/center/2067/Centre-Kawtar-de-Laval--3871-Autoroute-des-Laurentides,-Chomedey,-QC-H7L-3H7</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -797,16 +833,19 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>https://irizq.com/index.php/markaz-aicp-laval</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -844,21 +883,24 @@
           <t>438-788-0496</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
         <is>
           <t>https://jamiasiddiquialaval.com/</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>https://jamiasiddiquialaval.com/contact-us/</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -897,16 +939,19 @@
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>https://canada247.info/explore/quebec/laval/masjid-aljisr-450-681-2133.html</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -944,21 +989,24 @@
           <t>450-668-4381</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
         <is>
           <t>https://al-itissam.org/</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>https://prayersconnect.com/fr/mosques/12461611-masjid-al-itissam-laval-quebec-canada</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -996,21 +1044,24 @@
           <t>450-238-1402</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
         <is>
           <t>http://www.okba.org</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>https://esalah.com/mosques/canada/laval/laval/</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1045,16 +1096,19 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr">
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>https://praysalat.com/mosques/canada/quebec/laval</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1092,21 +1146,24 @@
           <t>514-802-3732</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
         <is>
           <t>https://amanlaval.com/</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>https://www.mosquee-proche.com/en/mosquee/centre-aman-laval/2025/</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1141,16 +1198,19 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>https://www.pagesjaunes.ca/search/si/1/Centre-Culturel-Islamique-De-Ste-Rose/Laval+QC</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1188,21 +1248,24 @@
           <t>450-256-0115</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
         <is>
           <t>https://centre-assalam.com/</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
         <is>
           <t>https://muslimguideme.com/en/place/Centre-Assalam-De-Laval-Est/1321</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1240,21 +1303,24 @@
           <t>438-396-6648</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
         <is>
           <t>https://www.essalam.ca</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>https://www.profilecanada.com/companydetail.cfm?company=719719_Centre_Communautaire_Musulman_Essalam_Mascouche_QC</t>
         </is>
       </c>
+      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1292,21 +1358,24 @@
           <t>450-932-3932</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
         <is>
           <t>https://ccilanaudiere.org/</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>https://www.lejournaldejoliette.ca/commerces/associations/46943/centre-culturel-islamique-de-lanaudiere</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1333,16 +1402,19 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr">
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>https://prayersconnect.com/mosques/12402132-masjid-terrebonne-sainte-julienne-quebec-canada</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1369,16 +1441,19 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr">
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>https://www.facebook.com/centrerayansaintetherese/</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1409,16 +1484,19 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>https://mawaqit.net/en/m/masjid-al-hak-saint-jerome-j7z-5m2-canada</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1457,16 +1535,19 @@
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>https://yably.ca/reviews/saint-jerome/mosquee-minaret-du-nord-293-rue-labelle</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1496,21 +1577,24 @@
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
         <is>
           <t>https://mosqueealfirdaws.net/</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
         <is>
           <t>https://mosqueealfirdaws.net/</t>
         </is>
       </c>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1549,16 +1633,19 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>https://proudmuslimmtl.ca/masjids/pierrefonds-roxboro/</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1597,16 +1684,19 @@
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
         <is>
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3152-centre-islamique-du-west-island?city=montreal</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1641,16 +1731,19 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>https://mapcarta.com/N6467166681</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1689,16 +1782,19 @@
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3154-al-khoei-mtl?city=Montreal</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1737,16 +1833,19 @@
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3126-baitul-mukkarram?city=montreal</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1785,16 +1884,19 @@
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3144-al-falah?city=Montreal</t>
         </is>
       </c>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1828,21 +1930,24 @@
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr">
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
         <is>
           <t>https://mosquee-dhoun-nourain.com/</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>https://mosquee-dhoun-nourain.com/contact/</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1877,16 +1982,19 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
         <is>
           <t>https://moonode.com/entity/taiba-410971-3560-avenue-van-horne-montreal-qc-h3s-1r6-canada</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1920,21 +2028,24 @@
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
         <is>
           <t>https://www.amlachine.org/en</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
         <is>
           <t>https://www.amlachine.org/en</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1972,21 +2083,24 @@
           <t>514-367-5858</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
         <is>
           <t>http://www.cmlasalle.org/</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>https://canada247.org/explore/quebec/communaute_urbaine_de_montreal/montreal/lasalle/musalla-umar.html</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2024,21 +2138,24 @@
           <t>514-545-2515</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
         <is>
           <t>ndg-mosque.com</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
         <is>
           <t>https://www.praysalat.com/mosque/montreal/2226-mosquee-ndg</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2072,21 +2189,24 @@
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr">
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
         <is>
           <t>https://muslimcommunityofquebec.ca/</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>https://islammessage.org/en/center/2058/Muslim-Community-of-Quebec--7445-Chester-Avenue,-NDG,-Montr%C3%A9al,-QC-H4V-1M4</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2124,21 +2244,24 @@
           <t>514-278-8441</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
         <is>
           <t>https://assuna.org/</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
         <is>
           <t>http://assuna.org/services-et-appui/mosquee/</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2177,16 +2300,19 @@
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
         <is>
           <t>https://proudmuslimmtl.ca/masjids/pierrefonds-roxboro/</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2225,16 +2351,19 @@
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
         <is>
           <t>https://proudmuslimmtl.ca/masjids/pierrefonds-roxboro/</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2272,21 +2401,24 @@
           <t>514-939-0681</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
         <is>
           <t>https://www.iqrafoundation.net/</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
         <is>
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3162-khadijah-masjid?city=montreal</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2324,21 +2456,24 @@
           <t>514-360-2360</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
         <is>
           <t>https://www.icandalous.ca/</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
         <is>
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3106-Al-Andalous?city=montreal</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2377,16 +2512,19 @@
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3158-centre-islamique-de-verdun?city=montreal</t>
         </is>
       </c>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2413,16 +2551,19 @@
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr">
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>https://www.salam-mosque.org/</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2449,16 +2590,19 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr">
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>https://www.icqmontreal.com/montrealMosques.html</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2488,21 +2632,24 @@
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr">
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
         <is>
           <t>https://www.salam-mosque.org/</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>https://www.salam-mosque.org/</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2533,16 +2680,19 @@
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr">
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>https://www.islamicfinder.org/world/view-place/60436/</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2580,21 +2730,24 @@
           <t>514-991-3441</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
         <is>
           <t>https://tawuba.ca/</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
         <is>
           <t>https://proudmuslimmtl.ca/masjids/mercier-hochelaga-maisonneuve/</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2628,21 +2781,24 @@
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr">
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
         <is>
           <t>http://www.mamoor.ca</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
         <is>
           <t>http://www.mamoor.ca/location.html</t>
         </is>
       </c>
+      <c r="M47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2677,16 +2833,19 @@
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
         <is>
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3151-salahouddine-mosque?city=montreal</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2724,21 +2883,24 @@
           <t>514-416-6244</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
         <is>
           <t>http://www.ammn.ca</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>https://proudmuslimmtl.ca/masjids/montreal-nord/</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2776,21 +2938,24 @@
           <t>514-852-0778</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
         <is>
           <t>http://achoura.ca</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
         <is>
           <t>https://www.yellowpages.ca/bus/Quebec/Montreal-Nord/Centre-Culturel-Islamique-Ach-Choura/7123192.html</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2829,16 +2994,19 @@
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
         <is>
           <t>https://moonode.com/entity/islamic-center-al-houda--828889-9935-av-lausanne-montreal-nord-qc-h1h-5a6-canada</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2876,21 +3044,24 @@
           <t>514-727-6666</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
         <is>
           <t>http://azzahra.ca</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
         <is>
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3180-fatima-azzahra?city=montreal</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2928,21 +3099,24 @@
           <t>514-508-5282</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
         <is>
           <t>http://www.imamwarch.com</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
         <is>
           <t>https://moonode.com/entity/imam-warch-813840-3210-boul-henri-bourassa-e-montreal-nord-qc-h1h-5t1-canada</t>
         </is>
       </c>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2980,21 +3154,24 @@
           <t>438-270-5089</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
         <is>
           <t>https://masjidcanada.org/</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr">
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
         <is>
           <t>https://masjidcanada.org/</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3029,16 +3206,19 @@
       </c>
       <c r="G55" t="inlineStr"/>
       <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr">
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="L55" t="inlineStr">
         <is>
           <t>https://www.scribd.com/doc/90596543/Liste-Mosque-Last</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3073,16 +3253,19 @@
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr">
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
         <is>
           <t>https://praysalat.com/mosque/montreal/47730-mosquee-et-centre-communautaire-ccsca</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3120,21 +3303,24 @@
           <t>514-951-1660</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
         <is>
           <t>http://www.elfath.ca/</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr">
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
         <is>
           <t>https://proudmuslimmtl.ca/masjids/riviere-des-prairies-pointe-aux-trembles/</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3173,16 +3359,19 @@
         </is>
       </c>
       <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr">
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
         <is>
           <t>https://proudmuslimmtl.ca/masjids/rosemont-le-petite-partie/</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3220,21 +3409,24 @@
           <t>514-725-0008</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
         <is>
           <t>http://cciem.org/</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
         <is>
           <t>https://www.pagesjaunes.ca/bus/Quebec/Montreal/Centre-Communautaire-Islamique-De-L-Est-De-Montr-eal/7497449.html</t>
         </is>
       </c>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3272,21 +3464,24 @@
           <t>514-255-6460</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
         <is>
           <t>http://www.centrebadr.net/</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr">
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
         <is>
           <t>https://proudmuslimmtl.ca/masjids/saint-leonard/</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3324,21 +3519,24 @@
           <t>514-552-3122</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
         <is>
           <t>https://www.centres-tawhid.ca/</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
         <is>
           <t>https://proudmuslimmtl.ca/masjids/saint-leonard/</t>
         </is>
       </c>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3376,21 +3574,24 @@
           <t>514-223-2353</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
         <is>
           <t>https://www.altawhid.ca/</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
         <is>
           <t>https://www.altawhid.ca/</t>
         </is>
       </c>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3425,16 +3626,19 @@
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="L63" t="inlineStr">
         <is>
           <t>https://proudmuslimmtl.ca/masjids/saint-leonard/</t>
         </is>
       </c>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3473,16 +3677,19 @@
         </is>
       </c>
       <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J64" t="inlineStr">
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>https://www.pagesjaunes.ca/bus/Quebec/Montreal/Centre-Et-Mosquee-Assalam/102188614.html</t>
         </is>
       </c>
+      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3521,16 +3728,19 @@
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J65" t="inlineStr">
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
         <is>
           <t>https://prayersconnect.com/mosques/12494853-turkish-islamic-center-of-quebec-montreal-quebec-canada</t>
         </is>
       </c>
+      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3568,21 +3778,24 @@
           <t>514-383-3682</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
         <is>
           <t>http://www.belagir.ca</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J66" t="inlineStr">
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
         <is>
           <t>https://moonode.com/entity/bel-agir-192280-8390-rue-st-hubert-montreal-qc-h2p-1z3-canada</t>
         </is>
       </c>
+      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3620,21 +3833,24 @@
           <t>514-506-8899</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr">
         <is>
           <t>https://ccvmac.ca</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J67" t="inlineStr">
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
         <is>
           <t>https://www.facebook.com/ccvmac.ca/</t>
         </is>
       </c>
+      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3672,21 +3888,24 @@
           <t>450-641-9876</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr">
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
         <is>
           <t>https://ccmboucherville.ca/</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
         <is>
           <t>https://ccmboucherville.ca/</t>
         </is>
       </c>
+      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3713,16 +3932,19 @@
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr">
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
+      <c r="L69" t="inlineStr">
         <is>
           <t>https://www.zabihah.com/mosques/cb660389-7767-11ef-95ae-6045bdeb9f57/abshar-brossard-qc</t>
         </is>
       </c>
+      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3757,16 +3979,19 @@
       </c>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr">
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
+      <c r="L70" t="inlineStr">
         <is>
           <t>https://salatomatic.com/spc/bC9P4EsQmF</t>
         </is>
       </c>
+      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3804,21 +4029,24 @@
           <t>450-656-9841</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr">
         <is>
           <t>https://iccbrossard.com/</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
         <is>
           <t>https://brossard-quebec.catalog-online.ca/mosque/islamic-community-center-brossard/</t>
         </is>
       </c>
+      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3852,21 +4080,24 @@
         </is>
       </c>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr">
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
         <is>
           <t>https://www.apchambly.com/</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr">
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
         <is>
           <t>https://islammessage.org/fr/center/2053/Association-de-la-Paix-de-Chambly--1691-Boulevard-de-P%C3%A9rigny,-Chambly,-QC-J3L-1X1</t>
         </is>
       </c>
+      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3900,21 +4131,24 @@
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr">
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr">
         <is>
           <t>https://acmac.ca/</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
         <is>
           <t>https://acmac.ca/fr/mosque</t>
         </is>
       </c>
+      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3952,21 +4186,24 @@
           <t>514-207-0613</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr">
         <is>
           <t>https://ccmchateauguay.org/</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
         <is>
           <t>https://www.waze.com/live-map/directions/ca/qc/chateauguay/centre-culturel-musulman-de-chateauguay-mosquee-arrahmane?to=place.ChIJX5xkjlAVyUwRlR-KUovIaF0</t>
         </is>
       </c>
+      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4000,21 +4237,24 @@
         </is>
       </c>
       <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr">
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr">
         <is>
           <t>https://mosqueechateauguay.ca/</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="K75" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="L75" t="inlineStr">
         <is>
           <t>https://mosqueechateauguay.ca/locations/mosquee-chateauguay/</t>
         </is>
       </c>
+      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4048,21 +4288,24 @@
         </is>
       </c>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr">
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr">
         <is>
           <t>https://masjidattawassol.com/</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
+      <c r="K76" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="L76" t="inlineStr">
         <is>
           <t>https://masjidattawassol.com/en/</t>
         </is>
       </c>
+      <c r="M76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4100,21 +4343,24 @@
           <t>450-321-1225</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr">
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr">
         <is>
           <t>https://ccmlongueuil.ca/</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
         <is>
           <t>https://opengovca.com/quebec-business/1164163843</t>
         </is>
       </c>
+      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4153,16 +4399,19 @@
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
         <is>
           <t>https://moonode.com/entity/jamia-islamia-498266-2144-rue-sainte-helene-longueuil-qc-j4k-3t6-canada</t>
         </is>
       </c>
+      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4197,16 +4446,19 @@
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr">
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr">
+      <c r="L79" t="inlineStr">
         <is>
           <t>https://www.yellowpages.ca/bus/Quebec/Saint-Constant/Centre-Musulman-Al-Manara/100866854.html</t>
         </is>
       </c>
+      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4244,21 +4496,24 @@
           <t>450-443-3482</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr">
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr">
         <is>
           <t>https://masjidalfalah.ca/</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr">
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
         <is>
           <t>https://moonode.com/entity/al-falah-longueuil-367873-1885-rue-nielsen-saint-hubert-qc-j4t-1p1-canada</t>
         </is>
       </c>
+      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4292,21 +4547,24 @@
         </is>
       </c>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr">
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr">
         <is>
           <t>https://cimaskoutain.com/</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J81" t="inlineStr">
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
         <is>
           <t>https://islammessage.org/en/center/2044/Centre-Islamique-Les-Maskoutains--2340-Avenue-Saint-Joseph,-Saint-Hyacinthe,-QC-J2S-5L5</t>
         </is>
       </c>
+      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4344,21 +4602,24 @@
           <t>450-800-4266</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr">
         <is>
           <t>https://ccai-stjean.org/</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J82" t="inlineStr">
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
         <is>
           <t>https://www.thehashir.com/mosques-details/Centre-Communautaire-Al-Imane/314</t>
         </is>
       </c>
+      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4397,16 +4658,19 @@
         </is>
       </c>
       <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J83" t="inlineStr">
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
         <is>
           <t>https://www.islamicfinder.org/world/view-place/55720/?language=fr</t>
         </is>
       </c>
+      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4432,21 +4696,24 @@
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr">
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr">
         <is>
           <t>http://www.ccmsoreltracy.ca/</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr">
+      <c r="K84" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr">
+      <c r="L84" t="inlineStr">
         <is>
           <t>https://mawaqit.net/en/m/ccm-sorel-tracy</t>
         </is>
       </c>
+      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4484,21 +4751,24 @@
           <t>450-218-3687</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr">
         <is>
           <t>https://www.islamvaudreuil.ca/</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
         <is>
           <t>https://canada247.info/explore/quebec/vaudreuil_soulanges/vaudreuil_dorion/dorion/centre-culturel-islamique-de-vaudreuil-soulanges-450-218-3687.html</t>
         </is>
       </c>
+      <c r="M85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4529,16 +4799,19 @@
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr">
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
+      <c r="K86" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr">
+      <c r="L86" t="inlineStr">
         <is>
           <t>https://td.maptons.com/p/1920918333</t>
         </is>
       </c>
+      <c r="M86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4568,21 +4841,24 @@
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr">
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+      <c r="J87" t="inlineStr">
         <is>
           <t>https://centreislamiquededrummondville.com/</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr">
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
         <is>
           <t>https://centreislamiquededrummondville.com/</t>
         </is>
       </c>
+      <c r="M87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4616,21 +4892,24 @@
         </is>
       </c>
       <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr">
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
         <is>
           <t>https://www.mosque-aylmer.ca/</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
         <is>
           <t>https://www.mosque-aylmer.ca/</t>
         </is>
       </c>
+      <c r="M88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4664,21 +4943,24 @@
         </is>
       </c>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr">
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr">
         <is>
           <t>https://cio-oic.ca/</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
         <is>
           <t>https://cio-oic.ca/locations/la-mosquee-de-gatineau/</t>
         </is>
       </c>
+      <c r="M89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4716,21 +4998,24 @@
           <t>450-994-3091</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr">
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr">
         <is>
           <t>https://mosqueegranby.com/</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
         <is>
           <t>https://islammessage.org/en/center/2074/Centre-Culturel-Islamique-de-Granby--317-Rue-Racine,-Granby,-QC-J2G-3B6</t>
         </is>
       </c>
+      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4764,21 +5049,24 @@
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr">
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr">
         <is>
           <t>https://ccilapoc.ca/</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr">
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
         <is>
           <t>https://ccilapoc.ca/</t>
         </is>
       </c>
+      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4816,21 +5104,24 @@
           <t>418-803-0212</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr">
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr">
         <is>
           <t>https://centreculturelammgl.ca/</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
         <is>
           <t>https://www.lesoleil.com/actualites/actualites-locales/la-capitale/2025/11/30/un-reve-devenu-realite-la-mosquee-de-levis-a-trouve-son-nouveau-toit-YC2SEX7YIJAK5PLFHEPLGTA3OQ/</t>
         </is>
       </c>
+      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4865,16 +5156,19 @@
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
         <is>
           <t>https://www.omradiscount.fr/mosquees/canada/magog/acim-magog-qc-j1x-1t5-canada</t>
         </is>
       </c>
+      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4913,16 +5207,19 @@
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
         <is>
           <t>https://islammessage.org/en/center/2104/Mosquee-Al-Rahma--363-Rue-de-la-Couronne,-Unit-301-302,-Quebec-City,-QC-G1K-6E9</t>
         </is>
       </c>
+      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4961,16 +5258,19 @@
         </is>
       </c>
       <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J95" t="inlineStr">
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
         <is>
           <t>https://www.yellowpages.ca/bus/Quebec/Quebec/Mosquee-De-La-Capitale/8113912.html</t>
         </is>
       </c>
+      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5004,21 +5304,24 @@
         </is>
       </c>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr">
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr">
         <is>
           <t>https://www.facebook.com/mosqueealathar/</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr">
+      <c r="K96" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr">
+      <c r="L96" t="inlineStr">
         <is>
           <t>https://mawaqit.net/en/m/masjid-al-athar-quebec-g1j-3b3-canada</t>
         </is>
       </c>
+      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5056,21 +5359,24 @@
           <t>418-473-4447</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr">
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr">
         <is>
           <t>http://www.mosqueedequebec.com/</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J97" t="inlineStr">
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
         <is>
           <t>https://fr.wikipedia.org/wiki/Mosqu%C3%A9e_de_Qu%C3%A9bec_%C3%A0_Limoilou</t>
         </is>
       </c>
+      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5104,21 +5410,24 @@
         </is>
       </c>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr">
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr">
         <is>
           <t>https://aemul.asso.ulaval.ca/</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr">
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
         <is>
           <t>https://therevertproject.org/masjidquebeccity</t>
         </is>
       </c>
+      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5156,21 +5465,24 @@
           <t>418-683-1329</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr">
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr">
         <is>
           <t>https://cciq.org/</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr">
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
         <is>
           <t>https://www.mosquee-proche.com/mosquee/cciq/2022/</t>
         </is>
       </c>
+      <c r="M99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5204,21 +5516,24 @@
         </is>
       </c>
       <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr">
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr">
         <is>
           <t>https://mawaqit.net/en/mosquee-de-rimouski-rimouski</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J100" t="inlineStr">
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
         <is>
           <t>https://www.mosquee-proche.com/fr/mosquee/mosquee-de-rimouski-rimouski/2018/</t>
         </is>
       </c>
+      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5252,21 +5567,24 @@
         </is>
       </c>
       <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr">
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr">
         <is>
           <t>https://association-socio-culturelle-islamique.business.site/</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J101" t="inlineStr">
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
         <is>
           <t>https://www.mosquee-proche.com/fr/mosquee/ascil-rdl-riviere-du-loup-g5r3a7-canada/4251/</t>
         </is>
       </c>
+      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5300,21 +5618,24 @@
         </is>
       </c>
       <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr">
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr">
         <is>
           <t>http://acmrn.org/</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J102" t="inlineStr">
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
         <is>
           <t>https://prayersconnect.com/mosques/12443730-mosquee-de-rouyn-noranda-rouyn-noranda-quebec-canada</t>
         </is>
       </c>
+      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5344,21 +5665,24 @@
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr">
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr">
         <is>
           <t>https://mawaqit.net/en/mosquee-chicoutimi</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J103" t="inlineStr">
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
         <is>
           <t>https://mawaqit.net/en/mosquee-chicoutimi</t>
         </is>
       </c>
+      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5392,21 +5716,24 @@
         </is>
       </c>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr">
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr">
         <is>
           <t>https://ccidelabeauce.ca/</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J104" t="inlineStr">
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
         <is>
           <t>https://mawaqit.net/en/cci-de-la-beauce-saint-georges-g5y-1v9-canada</t>
         </is>
       </c>
+      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5432,21 +5759,24 @@
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr">
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr">
         <is>
           <t>https://ccmcotenord.wixsite.com/ccmcn</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr">
+      <c r="K105" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr">
+      <c r="L105" t="inlineStr">
         <is>
           <t>https://iqna.ir/fr/news/3496693/la-mosquee-de-sept-iles-ouvre-ses-portes-et-fait-decouvrir-le-patrimoine-musulman</t>
         </is>
       </c>
+      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5476,21 +5806,24 @@
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr">
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr">
         <is>
           <t>http://ccmshawinigan.ca/</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J106" t="inlineStr">
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
         <is>
           <t>https://ici.radio-canada.ca/nouvelle/712529/mosquee-shawinigan-rue-saint-marc</t>
         </is>
       </c>
+      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5528,21 +5861,24 @@
           <t>819-481-1548</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr">
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr">
         <is>
           <t>https://www.ccis-annour.ca/</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr">
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
         <is>
           <t>https://canada247.info/explore/quebec/la_region_sherbrookoise/sherbrooke/jacques_cartier/mosque_annour.html</t>
         </is>
       </c>
+      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5576,21 +5912,24 @@
         </is>
       </c>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr">
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr">
         <is>
           <t>https://www.acie.ca/</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J108" t="inlineStr">
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
         <is>
           <t>https://mawaqit.net/en/mosquee-rahman-ctr-culturel-sherbrooke-qc</t>
         </is>
       </c>
+      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5616,21 +5955,24 @@
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr">
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@CentreculturelIslamique</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr">
+      <c r="K109" t="inlineStr">
         <is>
           <t>low</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr">
+      <c r="L109" t="inlineStr">
         <is>
           <t>https://www.facebook.com/p/Centre-Culturel-Islamique-61573929870434/</t>
         </is>
       </c>
+      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5664,21 +6006,24 @@
           <t>819-378-0419</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr">
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr">
         <is>
           <t>https://ccim3r.ca/</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J110" t="inlineStr">
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
         <is>
           <t>https://ccim3r.ca/histoire.html</t>
         </is>
       </c>
+      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5712,21 +6057,24 @@
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr">
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr">
         <is>
           <t>https://acmvaldor.org/</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J111" t="inlineStr">
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
         <is>
           <t>https://www.zabihah.com/mosques/1380a94a-776a-11ef-95ae-6045bdeb9f57/association-culturelle-musulmane-de-val-dor-val-d-or-qc</t>
         </is>
       </c>
+      <c r="M111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5760,21 +6108,24 @@
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr">
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr">
         <is>
           <t>https://acibf.org/</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="J112" t="inlineStr">
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
         <is>
           <t>https://prayersconnect.com/fr/mosques/12426349-islamic-cultural-association-of-bois-francs-victoriaville-quebec-canada</t>
         </is>
       </c>
+      <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5804,24 +6155,27 @@
       </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr">
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr">
         <is>
           <t>https://www.facebook.com/CentreCIV/</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr">
+      <c r="K113" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="J113" t="inlineStr">
+      <c r="L113" t="inlineStr">
         <is>
           <t>https://www.facebook.com/CentreCIV/</t>
         </is>
       </c>
+      <c r="M113" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J113"/>
+  <autoFilter ref="A1:M113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add contact emails to Quebec mosque list (66 of 112)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013QAvGezT92hRi1LAbYSDwT
</commit_message>
<xml_diff>
--- a/quebec-mosques/quebec_mosques.xlsx
+++ b/quebec-mosques/quebec_mosques.xlsx
@@ -546,8 +546,16 @@
           <t>450-750-0123</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>acmljoliette@gmail.com</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>info@acml-joliette.org</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>https://acml-joliette.org/</t>
@@ -563,7 +571,11 @@
           <t>https://prayersconnect.com/mosques/12412579-joliette-mosque-joliette-quebec-canada</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>https://acml-joliette.org/contact/</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -679,7 +691,11 @@
           <t>514-250-0265</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>contact@centreiqra.org</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
@@ -696,7 +712,11 @@
           <t>https://www.mosquee-proche.com/fr/mosquee/ccmi-centre-communautaire-musulman-iqra-laval-h7v-2v5-canada/5496/</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>https://centreiqra.org/</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -734,7 +754,11 @@
           <t>450-680-1612</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>contact@ccil-kbw.com</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
@@ -747,7 +771,11 @@
           <t>https://esalah.com/mosques/canada/laval/laval/</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>https://ccil-kbw.com/</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -785,7 +813,11 @@
           <t>450-682-8055</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>centrekawtar@outlook.com</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
@@ -798,7 +830,11 @@
           <t>https://islammessage.org/en/center/2067/Centre-Kawtar-de-Laval--3871-Autoroute-des-Laurentides,-Chomedey,-QC-H7L-3H7</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>https://centrekawtar.net/nous-joindre/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -883,8 +919,16 @@
           <t>438-788-0496</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>info@jamiasiddiquialaval.com</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>communitycentresiddiquia@gmail.com</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>https://jamiasiddiquialaval.com/</t>
@@ -900,7 +944,11 @@
           <t>https://jamiasiddiquialaval.com/contact-us/</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>https://jamiasiddiquialaval.com/contact-us/</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -938,7 +986,11 @@
           <t>450-681-2133</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>masjidaljisr@gmail.com</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
@@ -951,7 +1003,11 @@
           <t>https://canada247.info/explore/quebec/laval/masjid-aljisr-450-681-2133.html</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>https://centrealjisr.com/contacts/</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -989,7 +1045,11 @@
           <t>450-668-4381</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>info@al-itissam.org</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
@@ -1006,7 +1066,11 @@
           <t>https://prayersconnect.com/fr/mosques/12461611-masjid-al-itissam-laval-quebec-canada</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>https://al-itissam.org/contactez-nous/</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1146,7 +1210,11 @@
           <t>514-802-3732</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>masjid.alamane@gmail.com</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
@@ -1163,7 +1231,11 @@
           <t>https://www.mosquee-proche.com/en/mosquee/centre-aman-laval/2025/</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>https://www.mosquee-proche.com/en/mosquee/centre-aman-laval/2025/</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1248,8 +1320,16 @@
           <t>450-256-0115</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>centreassalam@gmail.com</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>info@centre-assalam.com</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr">
         <is>
           <t>https://centre-assalam.com/</t>
@@ -1265,7 +1345,11 @@
           <t>https://muslimguideme.com/en/place/Centre-Assalam-De-Laval-Est/1321</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>https://initiatives-musulmanes.com/dalilook/directory/centre-assalam-laval/</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1303,7 +1387,11 @@
           <t>438-396-6648</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>contact@essalam.ca</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
@@ -1320,7 +1408,11 @@
           <t>https://www.profilecanada.com/companydetail.cfm?company=719719_Centre_Communautaire_Musulman_Essalam_Mascouche_QC</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>https://www.essalam.ca/contact</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1358,7 +1450,11 @@
           <t>450-932-3932</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>communication@ccilanaudiere.org</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
@@ -1375,7 +1471,11 @@
           <t>https://www.lejournaldejoliette.ca/commerces/associations/46943/centre-culturel-islamique-de-lanaudiere</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>https://ccilanaudiere.org/</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1534,8 +1634,16 @@
           <t>450-821-3559</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>minaretdunord@gmail.com</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>info@manaratalchamal.org</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
@@ -1547,7 +1655,11 @@
           <t>https://yably.ca/reviews/saint-jerome/mosquee-minaret-du-nord-293-rue-labelle</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>https://minaretdunord.net/</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1577,7 +1689,11 @@
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>alfirdawsmasjid@gmail.com</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
@@ -1594,7 +1710,11 @@
           <t>https://mosqueealfirdaws.net/</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>https://mosqueealfirdaws.net/</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1632,7 +1752,11 @@
           <t>514-624-5833</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>cicaljamieh@gmail.com</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
@@ -1645,7 +1769,11 @@
           <t>https://proudmuslimmtl.ca/masjids/pierrefonds-roxboro/</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>http://cical-jamieh.com/en/contact-us/</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1683,7 +1811,11 @@
           <t>514-684-3100</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>info@icwestisland.com</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
@@ -1696,7 +1828,11 @@
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3152-centre-islamique-du-west-island?city=montreal</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>https://prayersconnect.com/mosques/12410160-islamic-center-of-west-island-dollard-des-ormeaux-quebec-canada/contact-us</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1730,7 +1866,11 @@
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>info@cclmac.ca</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
@@ -1743,7 +1883,11 @@
           <t>https://mapcarta.com/N6467166681</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>https://initiatives-musulmanes.com/dalilook/directory/mac-ccl/</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1781,8 +1925,16 @@
           <t>514-341-2235</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>info@khoei.ca</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>AlKhoeiFoundation@gmail.com</t>
+        </is>
+      </c>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
@@ -1794,7 +1946,11 @@
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3154-al-khoei-mtl?city=Montreal</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>https://www.khoei.ca/destinations</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1832,8 +1988,16 @@
           <t>514-737-8671</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>connect@mbmmtl.org</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>masjidbaitulmukarrammtl@gmail.com</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
@@ -1845,7 +2009,11 @@
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3126-baitul-mukkarram?city=montreal</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>https://initiatives-musulmanes.com/dalilook/directory/masjid-baitul-mukarram/</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2028,8 +2196,16 @@
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>contact@amlachine.org</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>info.aml.org@gmail.com</t>
+        </is>
+      </c>
       <c r="J32" t="inlineStr">
         <is>
           <t>https://www.amlachine.org/en</t>
@@ -2045,7 +2221,11 @@
           <t>https://www.amlachine.org/en</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>https://www.amlachine.org/en</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2138,7 +2318,11 @@
           <t>514-545-2515</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>info@ndg-mosque.com</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
@@ -2155,7 +2339,11 @@
           <t>https://www.praysalat.com/mosque/montreal/2226-mosquee-ndg</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>https://ndg-mosque.com/contact-us/</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2189,7 +2377,11 @@
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>info@muslimcommunityofquebec.ca</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
@@ -2206,7 +2398,11 @@
           <t>https://islammessage.org/en/center/2058/Muslim-Community-of-Quebec--7445-Chester-Avenue,-NDG,-Montr%C3%A9al,-QC-H4V-1M4</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>https://muslimcommunityofquebec.ca/contact/</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2244,7 +2440,11 @@
           <t>514-278-8441</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>assuna.annabawiyah@gmail.com</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
@@ -2261,7 +2461,11 @@
           <t>http://assuna.org/services-et-appui/mosquee/</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>http://assuna.org/contact-us/</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2299,7 +2503,11 @@
           <t>514-542-4832</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>admin@ccalhuda.ca</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
@@ -2312,7 +2520,11 @@
           <t>https://proudmuslimmtl.ca/masjids/pierrefonds-roxboro/</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>https://initiatives-musulmanes.com/dalilook/directory/masjid-al-huda/</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2350,7 +2562,11 @@
           <t>514-421-1455</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>masjidmakkah@outlook.com</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr">
@@ -2363,7 +2579,11 @@
           <t>https://proudmuslimmtl.ca/masjids/pierrefonds-roxboro/</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>https://masjidmakkah.com/contact-us/</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2401,7 +2621,11 @@
           <t>514-939-0681</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>info@khadijahmtl.org</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
@@ -2418,7 +2642,11 @@
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3162-khadijah-masjid?city=montreal</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>https://khadijahmtl.org/venue/khadijah-centre/</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2456,7 +2684,11 @@
           <t>514-360-2360</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>info@icandalous.ca</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
@@ -2473,7 +2705,11 @@
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3106-Al-Andalous?city=montreal</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>https://www.icandalous.ca/contactez-nous/</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2511,8 +2747,16 @@
           <t>514-508-9419</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>verdun.muslims@gmail.com</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>info@civmac.ca</t>
+        </is>
+      </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
@@ -2524,7 +2768,11 @@
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3158-centre-islamique-de-verdun?city=montreal</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3158-centre-islamique-de-verdun?city=montreal</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2550,7 +2798,11 @@
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>info@almadinah-center.org</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
@@ -2563,7 +2815,11 @@
           <t>https://www.salam-mosque.org/</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>https://almadinah-center.org/en/contact-us/</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2632,7 +2888,11 @@
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>info@salam-mosque.org</t>
+        </is>
+      </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
@@ -2649,7 +2909,11 @@
           <t>https://www.salam-mosque.org/</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>https://www.salam-mosque.org/prayer-times/</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2730,7 +2994,11 @@
           <t>514-991-3441</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>tawubamosque@gmail.com</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
@@ -2747,7 +3015,11 @@
           <t>https://proudmuslimmtl.ca/masjids/mercier-hochelaga-maisonneuve/</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>https://tawuba.ca/</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2781,7 +3053,11 @@
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>baitulmamoor@gmail.com</t>
+        </is>
+      </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
@@ -2798,7 +3074,11 @@
           <t>http://www.mamoor.ca/location.html</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3155-baitul-ma-moor?city=montreal</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2832,7 +3112,11 @@
           <t>514-274-6194</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>info@aicp.ca</t>
+        </is>
+      </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr">
@@ -2845,7 +3129,11 @@
           <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3151-salahouddine-mosque?city=montreal</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3151-salahouddine-mosque?city=montreal</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2883,7 +3171,11 @@
           <t>514-416-6244</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>info@ammn.ca</t>
+        </is>
+      </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
@@ -2900,7 +3192,11 @@
           <t>https://proudmuslimmtl.ca/masjids/montreal-nord/</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>https://ammn.ca/contact</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2938,7 +3234,11 @@
           <t>514-852-0778</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>c.c.achoura@gmail.com</t>
+        </is>
+      </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
@@ -2955,7 +3255,11 @@
           <t>https://www.yellowpages.ca/bus/Quebec/Montreal-Nord/Centre-Culturel-Islamique-Ach-Choura/7123192.html</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>https://achoura.ca/contactus</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3154,7 +3458,11 @@
           <t>438-270-5089</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>info@masjidcanada.org</t>
+        </is>
+      </c>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
@@ -3171,7 +3479,11 @@
           <t>https://masjidcanada.org/</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>https://masjidcanada.org/</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3303,7 +3615,11 @@
           <t>514-951-1660</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>ccf.rdp@gmail.com</t>
+        </is>
+      </c>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
@@ -3320,7 +3636,11 @@
           <t>https://proudmuslimmtl.ca/masjids/riviere-des-prairies-pointe-aux-trembles/</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr"/>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>https://initiatives-musulmanes.com/dalilook/directory/centre-communautaire-el-fath/</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3409,7 +3729,11 @@
           <t>514-725-0008</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>centre.ciem@gmail.com</t>
+        </is>
+      </c>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
@@ -3426,7 +3750,11 @@
           <t>https://www.pagesjaunes.ca/bus/Quebec/Montreal/Centre-Communautaire-Islamique-De-L-Est-De-Montr-eal/7497449.html</t>
         </is>
       </c>
-      <c r="M59" t="inlineStr"/>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>http://cciem.org/</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3464,7 +3792,11 @@
           <t>514-255-6460</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>info@centrebadr.net</t>
+        </is>
+      </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr">
         <is>
@@ -3481,7 +3813,11 @@
           <t>https://proudmuslimmtl.ca/masjids/saint-leonard/</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr"/>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>https://www.muslimguide.com/show/Centre_Islamique_Badr_4660</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3519,7 +3855,11 @@
           <t>514-552-3122</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>centres.tawhid@gmail.com</t>
+        </is>
+      </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
@@ -3536,7 +3876,11 @@
           <t>https://proudmuslimmtl.ca/masjids/saint-leonard/</t>
         </is>
       </c>
-      <c r="M61" t="inlineStr"/>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>https://www.centres-tawhid.ca/contact/</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3574,7 +3918,11 @@
           <t>514-223-2353</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>contact@altawheed.ca</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
@@ -3591,7 +3939,11 @@
           <t>https://www.altawhid.ca/</t>
         </is>
       </c>
-      <c r="M62" t="inlineStr"/>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>https://www.altawhid.ca/</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3727,7 +4079,11 @@
           <t>514-722-1835</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>info@turkcommunity.ca</t>
+        </is>
+      </c>
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr">
@@ -3740,7 +4096,11 @@
           <t>https://prayersconnect.com/mosques/12494853-turkish-islamic-center-of-quebec-montreal-quebec-canada</t>
         </is>
       </c>
-      <c r="M65" t="inlineStr"/>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>https://muslimlink.ca/directory/montreal/muslim-services/masjids-musallahs/3164-turkish-community-center?city=Montreal</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3778,7 +4138,11 @@
           <t>514-383-3682</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>centre.belagir.mtl@gmail.com</t>
+        </is>
+      </c>
       <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
@@ -3795,7 +4159,11 @@
           <t>https://moonode.com/entity/bel-agir-192280-8390-rue-st-hubert-montreal-qc-h2p-1z3-canada</t>
         </is>
       </c>
-      <c r="M66" t="inlineStr"/>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>https://centre-belagir.ca/</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3833,7 +4201,11 @@
           <t>514-506-8899</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>info@ccvmac.ca</t>
+        </is>
+      </c>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
@@ -3850,7 +4222,11 @@
           <t>https://www.facebook.com/ccvmac.ca/</t>
         </is>
       </c>
-      <c r="M67" t="inlineStr"/>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>https://mawaqit.net/en/ccvmac-montreal</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4029,7 +4405,11 @@
           <t>450-656-9841</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>services@iccbrossard.com</t>
+        </is>
+      </c>
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
@@ -4046,7 +4426,11 @@
           <t>https://brossard-quebec.catalog-online.ca/mosque/islamic-community-center-brossard/</t>
         </is>
       </c>
-      <c r="M71" t="inlineStr"/>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>https://iccbrossard.com/</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4080,7 +4464,11 @@
         </is>
       </c>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>info@apchambly.com</t>
+        </is>
+      </c>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
@@ -4097,7 +4485,11 @@
           <t>https://islammessage.org/fr/center/2053/Association-de-la-Paix-de-Chambly--1691-Boulevard-de-P%C3%A9rigny,-Chambly,-QC-J3L-1X1</t>
         </is>
       </c>
-      <c r="M72" t="inlineStr"/>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>https://apchambly.com/contact.html</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4131,7 +4523,11 @@
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>sadaqa@acmac.ca</t>
+        </is>
+      </c>
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
@@ -4148,7 +4544,11 @@
           <t>https://acmac.ca/fr/mosque</t>
         </is>
       </c>
-      <c r="M73" t="inlineStr"/>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>https://www.acmac.ca/fr</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4186,7 +4586,11 @@
           <t>514-207-0613</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>razmane24@gmail.com</t>
+        </is>
+      </c>
       <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr">
         <is>
@@ -4203,7 +4607,11 @@
           <t>https://www.waze.com/live-map/directions/ca/qc/chateauguay/centre-culturel-musulman-de-chateauguay-mosquee-arrahmane?to=place.ChIJX5xkjlAVyUwRlR-KUovIaF0</t>
         </is>
       </c>
-      <c r="M74" t="inlineStr"/>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>https://prayersconnect.com/mosques/12461409-centre-culturel-musulman-de-chateauguay-mosquee-arrahmane-chateauguay-quebec-canada</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4288,8 +4696,16 @@
         </is>
       </c>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>info@cciroussillon.com</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>ccir@hotmail.com</t>
+        </is>
+      </c>
       <c r="J76" t="inlineStr">
         <is>
           <t>https://masjidattawassol.com/</t>
@@ -4305,7 +4721,11 @@
           <t>https://masjidattawassol.com/en/</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr"/>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>https://cciroussillon.com/</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4343,7 +4763,11 @@
           <t>450-321-1225</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>infoccmlongueuil@gmail.com</t>
+        </is>
+      </c>
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
@@ -4360,7 +4784,11 @@
           <t>https://opengovca.com/quebec-business/1164163843</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr"/>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>https://ccmlongueuil.ca/Contact.html</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4496,8 +4924,16 @@
           <t>450-443-3482</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>info@masjidalfalah.ca</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>donations@masjidalfalah.ca</t>
+        </is>
+      </c>
       <c r="J80" t="inlineStr">
         <is>
           <t>https://masjidalfalah.ca/</t>
@@ -4513,7 +4949,11 @@
           <t>https://moonode.com/entity/al-falah-longueuil-367873-1885-rue-nielsen-saint-hubert-qc-j4t-1p1-canada</t>
         </is>
       </c>
-      <c r="M80" t="inlineStr"/>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>https://masjidalfalah.ca/en/contact/</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4547,7 +4987,11 @@
         </is>
       </c>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>info@cimaskoutain.com</t>
+        </is>
+      </c>
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr">
         <is>
@@ -4564,7 +5008,11 @@
           <t>https://islammessage.org/en/center/2044/Centre-Islamique-Les-Maskoutains--2340-Avenue-Saint-Joseph,-Saint-Hyacinthe,-QC-J2S-5L5</t>
         </is>
       </c>
-      <c r="M81" t="inlineStr"/>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>https://cimaskoutain.com/contact/</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4602,7 +5050,11 @@
           <t>450-800-4266</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>centre.culturel.alimane.stjean@gmail.com</t>
+        </is>
+      </c>
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr">
         <is>
@@ -4619,7 +5071,11 @@
           <t>https://www.thehashir.com/mosques-details/Centre-Communautaire-Al-Imane/314</t>
         </is>
       </c>
-      <c r="M82" t="inlineStr"/>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>https://ccai-stjean.org/contactez-nous/</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4751,7 +5207,11 @@
           <t>450-218-3687</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>info-iccvs@islamvaudreuil.ca</t>
+        </is>
+      </c>
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr">
         <is>
@@ -4768,7 +5228,11 @@
           <t>https://canada247.info/explore/quebec/vaudreuil_soulanges/vaudreuil_dorion/dorion/centre-culturel-islamique-de-vaudreuil-soulanges-450-218-3687.html</t>
         </is>
       </c>
-      <c r="M85" t="inlineStr"/>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>https://www.islamvaudreuil.ca/contact</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4798,7 +5262,11 @@
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>ccmd.drummondville@gmail.com</t>
+        </is>
+      </c>
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr">
@@ -4811,7 +5279,11 @@
           <t>https://td.maptons.com/p/1920918333</t>
         </is>
       </c>
-      <c r="M86" t="inlineStr"/>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>http://www.ccmdrummond.com/nous_joindre.php</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4841,8 +5313,16 @@
       </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>centreislamiquedrummondville@hotmail.com</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>cidrummondville@gmail.com</t>
+        </is>
+      </c>
       <c r="J87" t="inlineStr">
         <is>
           <t>https://centreislamiquededrummondville.com/</t>
@@ -4858,7 +5338,11 @@
           <t>https://centreislamiquededrummondville.com/</t>
         </is>
       </c>
-      <c r="M87" t="inlineStr"/>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>https://centreislamiquededrummondville.com/</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4892,8 +5376,16 @@
         </is>
       </c>
       <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>info@mosque-aylmer.ca</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>finance@mosque-aylmer.ca</t>
+        </is>
+      </c>
       <c r="J88" t="inlineStr">
         <is>
           <t>https://www.mosque-aylmer.ca/</t>
@@ -4909,7 +5401,11 @@
           <t>https://www.mosque-aylmer.ca/</t>
         </is>
       </c>
-      <c r="M88" t="inlineStr"/>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>https://www.mosque-aylmer.ca/contact</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4943,7 +5439,11 @@
         </is>
       </c>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>info@cio-oic.ca</t>
+        </is>
+      </c>
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr">
         <is>
@@ -4960,7 +5460,11 @@
           <t>https://cio-oic.ca/locations/la-mosquee-de-gatineau/</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr"/>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>https://muslimlink.ca/directory/ottawa/muslim-services/masjids-musallahs/208-outaouais-islamic-centre-masjid-gatineau?city=ottawa</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4998,7 +5502,11 @@
           <t>450-994-3091</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>info@mosqueegranby.com</t>
+        </is>
+      </c>
       <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr">
         <is>
@@ -5015,7 +5523,11 @@
           <t>https://islammessage.org/en/center/2074/Centre-Culturel-Islamique-de-Granby--317-Rue-Racine,-Granby,-QC-J2G-3B6</t>
         </is>
       </c>
-      <c r="M90" t="inlineStr"/>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>https://mosqueegranby.com/</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5257,7 +5769,11 @@
           <t>418-914-2025</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>info@mosqueedelacapitale.com</t>
+        </is>
+      </c>
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr">
@@ -5270,7 +5786,11 @@
           <t>https://www.yellowpages.ca/bus/Quebec/Quebec/Mosquee-De-La-Capitale/8113912.html</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr"/>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>https://www.mosqueedelacapitale.com/nous-joindre/</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5304,7 +5824,11 @@
         </is>
       </c>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>salafisdequebec@hotmail.com</t>
+        </is>
+      </c>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr">
         <is>
@@ -5321,7 +5845,11 @@
           <t>https://mawaqit.net/en/m/masjid-al-athar-quebec-g1j-3b3-canada</t>
         </is>
       </c>
-      <c r="M96" t="inlineStr"/>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>https://prayersconnect.com/mosques/12453931-mosquee-al-athar-quebec-quebec-canada/contact-us</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5410,7 +5938,11 @@
         </is>
       </c>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>aemul@asso.ulaval.ca</t>
+        </is>
+      </c>
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr">
         <is>
@@ -5427,7 +5959,11 @@
           <t>https://therevertproject.org/masjidquebeccity</t>
         </is>
       </c>
-      <c r="M98" t="inlineStr"/>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>https://www.dse.ulaval.ca/association/association-des-etudiantes-musulmanes-de-l-universite-laval/</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5665,7 +6201,11 @@
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>mosqueechicoutimi2021@gmail.com</t>
+        </is>
+      </c>
       <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr">
         <is>
@@ -5682,7 +6222,11 @@
           <t>https://mawaqit.net/en/mosquee-chicoutimi</t>
         </is>
       </c>
-      <c r="M103" t="inlineStr"/>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/p/Association-Islamique-du-Saguenay-Lac-Saint-Jean-100080373907152/</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5861,8 +6405,16 @@
           <t>819-481-1548</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>contact@ccis-annour.ca</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>imam@ccis-annour.ca</t>
+        </is>
+      </c>
       <c r="J107" t="inlineStr">
         <is>
           <t>https://www.ccis-annour.ca/</t>
@@ -5878,7 +6430,11 @@
           <t>https://canada247.info/explore/quebec/la_region_sherbrookoise/sherbrooke/jacques_cartier/mosque_annour.html</t>
         </is>
       </c>
-      <c r="M107" t="inlineStr"/>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>https://www.ccis-annour.ca/contactez-nous</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5912,7 +6468,11 @@
         </is>
       </c>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>contact@acie.ca</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr">
         <is>
@@ -5929,7 +6489,11 @@
           <t>https://mawaqit.net/en/mosquee-rahman-ctr-culturel-sherbrooke-qc</t>
         </is>
       </c>
-      <c r="M108" t="inlineStr"/>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>https://www.acie.ca/en/contact</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6006,7 +6570,11 @@
           <t>819-378-0419</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>contact@ccim3r.ca</t>
+        </is>
+      </c>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr">
         <is>
@@ -6023,7 +6591,11 @@
           <t>https://ccim3r.ca/histoire.html</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr"/>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>https://ccim3r.ca/</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6057,7 +6629,11 @@
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>acmv.qc.ca@gmail.com</t>
+        </is>
+      </c>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr">
         <is>
@@ -6074,7 +6650,11 @@
           <t>https://www.zabihah.com/mosques/1380a94a-776a-11ef-95ae-6045bdeb9f57/association-culturelle-musulmane-de-val-dor-val-d-or-qc</t>
         </is>
       </c>
-      <c r="M111" t="inlineStr"/>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>https://acmvaldor.org/contact-2/</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">

</xml_diff>

<commit_message>
Split website-scraped emails into their own raw file (109 of 187 with email)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013QAvGezT92hRi1LAbYSDwT
</commit_message>
<xml_diff>
--- a/quebec-mosques/quebec_mosques.xlsx
+++ b/quebec-mosques/quebec_mosques.xlsx
@@ -5733,7 +5733,11 @@
           <t>don@cdsbalimaya.org</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>rahma@cdsbalimaya.org</t>
+        </is>
+      </c>
       <c r="J96" t="inlineStr">
         <is>
           <t>https://cdsbalimaya.org/</t>
@@ -8867,7 +8871,11 @@
           <t>info@civmac.ca</t>
         </is>
       </c>
-      <c r="I150" t="inlineStr"/>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>info@civmac.ca</t>
+        </is>
+      </c>
       <c r="J150" t="inlineStr">
         <is>
           <t>http://civmac.ca</t>
@@ -10800,8 +10808,16 @@
         </is>
       </c>
       <c r="G184" t="inlineStr"/>
-      <c r="H184" t="inlineStr"/>
-      <c r="I184" t="inlineStr"/>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>info@cio-oic.ca</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>imam@cio-oic.ca</t>
+        </is>
+      </c>
       <c r="J184" t="inlineStr">
         <is>
           <t>https://cio-oic.ca</t>
@@ -10817,7 +10833,11 @@
           <t>https://mawaqit.net/fr/cio-meriam</t>
         </is>
       </c>
-      <c r="M184" t="inlineStr"/>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>https://cio-oic.ca/contact-us</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">

</xml_diff>

<commit_message>
Add BCC list and prefer general inboxes over donation/IT addresses
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013QAvGezT92hRi1LAbYSDwT
</commit_message>
<xml_diff>
--- a/quebec-mosques/quebec_mosques.xlsx
+++ b/quebec-mosques/quebec_mosques.xlsx
@@ -6162,12 +6162,12 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
+          <t>rahma@cdsbalimaya.org</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
           <t>don@cdsbalimaya.org</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>rahma@cdsbalimaya.org</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -7998,12 +7998,12 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
+          <t>president@muslimcommunityofquebec.ca</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
           <t>IT@MuslimCommunityOfQuebec.ca</t>
-        </is>
-      </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>president@muslimcommunityofquebec.ca</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -11642,12 +11642,12 @@
       </c>
       <c r="H185" t="inlineStr">
         <is>
+          <t>imam@cio-oic.ca</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
           <t>display@cio-oic.ca</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr">
-        <is>
-          <t>imam@cio-oic.ca</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">

</xml_diff>

<commit_message>
Tag Salafi orgs and drop them and campus prayer rooms from the BCC list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013QAvGezT92hRi1LAbYSDwT
</commit_message>
<xml_diff>
--- a/quebec-mosques/quebec_mosques.xlsx
+++ b/quebec-mosques/quebec_mosques.xlsx
@@ -1205,7 +1205,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Mosque / centre</t>
+          <t>Salafi</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -4377,7 +4377,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Mosque / centre</t>
+          <t>Salafi</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7129,7 +7129,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Mosque / centre</t>
+          <t>Salafi</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -8333,7 +8333,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Mosque / centre</t>
+          <t>Salafi</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">

</xml_diff>